<commit_message>
feat(demo): refresh PANW pipeline outputs — forecasts, bundle, dashboard CSVs
Re-run of full demo pipeline: fact_forecasts now populated (12 rows),
NotebookLM bundle updated with latest forecast summary and eval report,
Excel model and Tableau CSVs regenerated from latest warehouse.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/PANW_3Statement_Model.xlsx
+++ b/dashboard/PANW_3Statement_Model.xlsx
@@ -197,8 +197,8 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="3" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="8" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -607,7 +607,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-22</t>
+          <t>Generated: 2026-05-24</t>
         </is>
       </c>
     </row>
@@ -811,13 +811,13 @@
         </is>
       </c>
       <c r="B2" s="6" t="n">
-        <v>0.04</v>
+        <v>-0.2</v>
       </c>
       <c r="C2" s="6" t="n">
-        <v>0.06</v>
+        <v>-0.3</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>0.016</v>
+        <v>-0.08000000000000002</v>
       </c>
     </row>
     <row r="3">
@@ -827,13 +827,13 @@
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>0.7377161055505005</v>
+        <v>0.68</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>0.7524704276615105</v>
+        <v>0.6936000000000001</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>0.7229617834394905</v>
+        <v>0.6664</v>
       </c>
     </row>
     <row r="4">
@@ -875,13 +875,13 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>43.32120109190173</v>
+        <v>60</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>41.15514103730664</v>
+        <v>57</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>47.65332120109191</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7">
@@ -891,13 +891,13 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>20.45099739809194</v>
+        <v>45</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>20.45099739809194</v>
+        <v>45</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>20.45099739809194</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8">
@@ -955,13 +955,13 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>0</v>
+        <v>615000000</v>
       </c>
       <c r="C11" s="8" t="n">
-        <v>0</v>
+        <v>615000000</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>0</v>
+        <v>615000000</v>
       </c>
     </row>
     <row r="12">
@@ -1042,7 +1042,7 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>0.04</v>
+        <v>-0.2</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -1057,7 +1057,7 @@
         </is>
       </c>
       <c r="B4" s="12" t="n">
-        <v>0.7377161055505005</v>
+        <v>0.68</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -1102,7 +1102,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>43.32120109190173</v>
+        <v>60</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -1117,7 +1117,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>20.45099739809194</v>
+        <v>45</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="B12" s="14" t="n">
-        <v>0</v>
+        <v>615000000</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
@@ -1331,37 +1331,41 @@
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B2" s="16" t="n"/>
-      <c r="C2" s="16" t="n"/>
-      <c r="D2" s="17" t="n">
+      <c r="B2" s="16" t="n">
+        <v>6685200000</v>
+      </c>
+      <c r="C2" s="16" t="n">
+        <v>5838000000</v>
+      </c>
+      <c r="D2" s="16" t="n">
+        <v>2139000000</v>
+      </c>
+      <c r="E2" s="16" t="n">
         <v>2474000000</v>
       </c>
-      <c r="E2" s="16" t="n"/>
-      <c r="F2" s="16" t="n"/>
-      <c r="G2" s="17" t="n">
-        <v>2139000000</v>
-      </c>
-      <c r="H2" s="16" t="n"/>
-      <c r="I2" s="16" t="n"/>
-      <c r="J2" s="16" t="n"/>
-      <c r="K2" s="17" t="n">
+      <c r="F2" s="17" t="n"/>
+      <c r="G2" s="17" t="n"/>
+      <c r="H2" s="17" t="n"/>
+      <c r="I2" s="16" t="n">
         <v>5068000000</v>
       </c>
-      <c r="L2" s="16" t="n"/>
-      <c r="M2" s="17" t="n">
+      <c r="J2" s="17" t="n"/>
+      <c r="K2" s="17" t="n"/>
+      <c r="L2" s="16" t="n">
         <v>4396000000</v>
       </c>
+      <c r="M2" s="17" t="n"/>
       <c r="N2" s="18" t="n">
-        <v>4571840000</v>
+        <v>0</v>
       </c>
       <c r="O2" s="18" t="n">
-        <v>4754713600</v>
+        <v>0</v>
       </c>
       <c r="P2" s="18" t="n">
-        <v>4944902144</v>
+        <v>0</v>
       </c>
       <c r="Q2" s="18" t="n">
-        <v>5142698229.76</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1370,37 +1374,41 @@
           <t>Cost of Revenue</t>
         </is>
       </c>
-      <c r="B3" s="16" t="n"/>
-      <c r="C3" s="16" t="n"/>
-      <c r="D3" s="17" t="n">
+      <c r="B3" s="16" t="n">
+        <v>1772600000</v>
+      </c>
+      <c r="C3" s="16" t="n">
+        <v>1485500000</v>
+      </c>
+      <c r="D3" s="16" t="n">
+        <v>554000000</v>
+      </c>
+      <c r="E3" s="16" t="n">
         <v>638000000</v>
       </c>
-      <c r="E3" s="16" t="n"/>
-      <c r="F3" s="16" t="n"/>
-      <c r="G3" s="17" t="n">
-        <v>554000000</v>
-      </c>
-      <c r="H3" s="16" t="n"/>
-      <c r="I3" s="16" t="n"/>
-      <c r="J3" s="16" t="n"/>
-      <c r="K3" s="17" t="n">
+      <c r="F3" s="17" t="n"/>
+      <c r="G3" s="17" t="n"/>
+      <c r="H3" s="17" t="n"/>
+      <c r="I3" s="16" t="n">
         <v>1323000000</v>
       </c>
-      <c r="L3" s="16" t="n"/>
-      <c r="M3" s="17" t="n">
+      <c r="J3" s="17" t="n"/>
+      <c r="K3" s="17" t="n"/>
+      <c r="L3" s="16" t="n">
         <v>1153000000</v>
       </c>
+      <c r="M3" s="17" t="n"/>
       <c r="N3" s="18" t="n">
-        <v>1199120000</v>
+        <v>0</v>
       </c>
       <c r="O3" s="18" t="n">
-        <v>1247084800</v>
+        <v>0</v>
       </c>
       <c r="P3" s="18" t="n">
-        <v>1296968192</v>
+        <v>0</v>
       </c>
       <c r="Q3" s="18" t="n">
-        <v>1348846919.68</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1409,37 +1417,41 @@
           <t>Gross Profit</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n"/>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="17" t="n">
+      <c r="B4" s="16" t="n">
+        <v>4912600000</v>
+      </c>
+      <c r="C4" s="16" t="n">
+        <v>4352500000</v>
+      </c>
+      <c r="D4" s="16" t="n">
+        <v>1585000000</v>
+      </c>
+      <c r="E4" s="16" t="n">
         <v>1836000000</v>
       </c>
-      <c r="E4" s="16" t="n"/>
-      <c r="F4" s="16" t="n"/>
-      <c r="G4" s="17" t="n">
-        <v>1585000000</v>
-      </c>
-      <c r="H4" s="16" t="n"/>
-      <c r="I4" s="16" t="n"/>
-      <c r="J4" s="16" t="n"/>
-      <c r="K4" s="17" t="n">
+      <c r="F4" s="17" t="n"/>
+      <c r="G4" s="17" t="n"/>
+      <c r="H4" s="17" t="n"/>
+      <c r="I4" s="16" t="n">
         <v>3745000000</v>
       </c>
-      <c r="L4" s="16" t="n"/>
-      <c r="M4" s="17" t="n">
+      <c r="J4" s="17" t="n"/>
+      <c r="K4" s="17" t="n"/>
+      <c r="L4" s="16" t="n">
         <v>3243000000</v>
       </c>
+      <c r="M4" s="17" t="n"/>
       <c r="N4" s="18" t="n">
-        <v>3372720000</v>
+        <v>0</v>
       </c>
       <c r="O4" s="18" t="n">
-        <v>3507628800</v>
+        <v>0</v>
       </c>
       <c r="P4" s="18" t="n">
-        <v>3647933952</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="18" t="n">
-        <v>3793851310.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1448,37 +1460,41 @@
           <t>Operating Expenses</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n"/>
-      <c r="C5" s="16" t="n"/>
-      <c r="D5" s="17" t="n">
+      <c r="B5" s="16" t="n">
+        <v>4166900000</v>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>3907000000</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>1299000000</v>
+      </c>
+      <c r="E5" s="16" t="n">
         <v>1527000000</v>
       </c>
-      <c r="E5" s="16" t="n"/>
-      <c r="F5" s="16" t="n"/>
-      <c r="G5" s="17" t="n">
-        <v>1299000000</v>
-      </c>
-      <c r="H5" s="16" t="n"/>
-      <c r="I5" s="16" t="n"/>
-      <c r="J5" s="16" t="n"/>
-      <c r="K5" s="17" t="n">
+      <c r="F5" s="17" t="n"/>
+      <c r="G5" s="17" t="n"/>
+      <c r="H5" s="17" t="n"/>
+      <c r="I5" s="16" t="n">
         <v>3039000000</v>
       </c>
-      <c r="L5" s="16" t="n"/>
-      <c r="M5" s="17" t="n">
+      <c r="J5" s="17" t="n"/>
+      <c r="K5" s="17" t="n"/>
+      <c r="L5" s="16" t="n">
         <v>2716000000</v>
       </c>
+      <c r="M5" s="17" t="n"/>
       <c r="N5" s="18" t="n">
-        <v>2172800000</v>
+        <v>0</v>
       </c>
       <c r="O5" s="18" t="n">
-        <v>1738240000</v>
+        <v>0</v>
       </c>
       <c r="P5" s="18" t="n">
-        <v>1390592000</v>
+        <v>0</v>
       </c>
       <c r="Q5" s="18" t="n">
-        <v>1112473600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1487,37 +1503,41 @@
           <t>Operating Income</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n"/>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="17" t="n">
+      <c r="B6" s="16" t="n">
+        <v>745700000</v>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>445500000</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>286000000</v>
+      </c>
+      <c r="E6" s="16" t="n">
         <v>309000000</v>
       </c>
-      <c r="E6" s="16" t="n"/>
-      <c r="F6" s="16" t="n"/>
-      <c r="G6" s="17" t="n">
-        <v>286000000</v>
-      </c>
-      <c r="H6" s="16" t="n"/>
-      <c r="I6" s="16" t="n"/>
-      <c r="J6" s="16" t="n"/>
-      <c r="K6" s="17" t="n">
+      <c r="F6" s="17" t="n"/>
+      <c r="G6" s="17" t="n"/>
+      <c r="H6" s="17" t="n"/>
+      <c r="I6" s="16" t="n">
         <v>706000000</v>
       </c>
-      <c r="L6" s="16" t="n"/>
-      <c r="M6" s="17" t="n">
+      <c r="J6" s="17" t="n"/>
+      <c r="K6" s="17" t="n"/>
+      <c r="L6" s="16" t="n">
         <v>527000000</v>
       </c>
+      <c r="M6" s="17" t="n"/>
       <c r="N6" s="18" t="n">
-        <v>1199920000</v>
+        <v>0</v>
       </c>
       <c r="O6" s="18" t="n">
-        <v>1769388800</v>
+        <v>0</v>
       </c>
       <c r="P6" s="18" t="n">
-        <v>2257341952</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="18" t="n">
-        <v>2681377710.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1526,37 +1546,41 @@
           <t>Net Income</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n"/>
-      <c r="C7" s="16" t="n"/>
-      <c r="D7" s="17" t="n">
+      <c r="B7" s="16" t="n">
+        <v>880100000</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>2219900000</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>351000000</v>
+      </c>
+      <c r="E7" s="16" t="n">
         <v>334000000</v>
       </c>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="16" t="n"/>
-      <c r="G7" s="17" t="n">
-        <v>351000000</v>
-      </c>
-      <c r="H7" s="16" t="n"/>
-      <c r="I7" s="16" t="n"/>
-      <c r="J7" s="16" t="n"/>
-      <c r="K7" s="17" t="n">
+      <c r="F7" s="17" t="n"/>
+      <c r="G7" s="17" t="n"/>
+      <c r="H7" s="17" t="n"/>
+      <c r="I7" s="16" t="n">
         <v>766000000</v>
       </c>
-      <c r="L7" s="16" t="n"/>
-      <c r="M7" s="17" t="n">
+      <c r="J7" s="17" t="n"/>
+      <c r="K7" s="17" t="n"/>
+      <c r="L7" s="16" t="n">
         <v>618000000</v>
       </c>
+      <c r="M7" s="17" t="n"/>
       <c r="N7" s="18" t="n">
-        <v>1019932000</v>
+        <v>0</v>
       </c>
       <c r="O7" s="18" t="n">
-        <v>1503980480</v>
+        <v>0</v>
       </c>
       <c r="P7" s="18" t="n">
-        <v>1918740659.2</v>
+        <v>0</v>
       </c>
       <c r="Q7" s="18" t="n">
-        <v>2279171053.568</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1565,29 +1589,35 @@
           <t>Gross Margin %</t>
         </is>
       </c>
+      <c r="B9" s="19" t="n">
+        <v>0.7348471249925208</v>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>0.7455464200068517</v>
+      </c>
       <c r="D9" s="19" t="n">
+        <v>0.7410004675081814</v>
+      </c>
+      <c r="E9" s="19" t="n">
         <v>0.7421180274858529</v>
       </c>
-      <c r="G9" s="19" t="n">
-        <v>0.7410004675081814</v>
-      </c>
-      <c r="K9" s="19" t="n">
+      <c r="I9" s="19" t="n">
         <v>0.738950276243094</v>
       </c>
-      <c r="M9" s="19" t="n">
+      <c r="L9" s="19" t="n">
         <v>0.7377161055505005</v>
       </c>
       <c r="N9" s="20" t="n">
-        <v>0.7377161055505005</v>
+        <v>0</v>
       </c>
       <c r="O9" s="20" t="n">
-        <v>0.7377161055505005</v>
+        <v>0</v>
       </c>
       <c r="P9" s="20" t="n">
-        <v>0.7377161055505005</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="20" t="n">
-        <v>0.7377161055505005</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1715,49 +1745,49 @@
           <t>Cash &amp; Equivalents</t>
         </is>
       </c>
-      <c r="B3" s="16" t="n"/>
-      <c r="C3" s="16" t="n"/>
-      <c r="D3" s="17" t="n">
+      <c r="B3" s="17" t="n"/>
+      <c r="C3" s="17" t="n"/>
+      <c r="D3" s="16" t="n">
         <v>2067200000</v>
       </c>
-      <c r="E3" s="17" t="n">
+      <c r="E3" s="16" t="n">
         <v>1346300000</v>
       </c>
-      <c r="F3" s="17" t="n">
+      <c r="F3" s="16" t="n">
+        <v>2118500000</v>
+      </c>
+      <c r="G3" s="16" t="n">
         <v>1992900000</v>
       </c>
-      <c r="G3" s="17" t="n">
-        <v>2118500000</v>
-      </c>
-      <c r="H3" s="17" t="n">
+      <c r="H3" s="16" t="n">
         <v>1373700000</v>
       </c>
-      <c r="I3" s="17" t="n">
+      <c r="I3" s="16" t="n">
         <v>2383400000</v>
       </c>
-      <c r="J3" s="17" t="n">
+      <c r="J3" s="16" t="n">
+        <v>3066000000</v>
+      </c>
+      <c r="K3" s="16" t="n">
         <v>2269000000</v>
       </c>
-      <c r="K3" s="17" t="n">
-        <v>3066000000</v>
-      </c>
-      <c r="L3" s="17" t="n">
+      <c r="L3" s="16" t="n">
         <v>2269000000</v>
       </c>
-      <c r="M3" s="17" t="n">
+      <c r="M3" s="16" t="n">
         <v>4158000000</v>
       </c>
       <c r="N3" s="18" t="n">
-        <v>5099200160</v>
+        <v>6798000000</v>
       </c>
       <c r="O3" s="18" t="n">
-        <v>6521299526.4</v>
+        <v>7584000000</v>
       </c>
       <c r="P3" s="18" t="n">
-        <v>8354883827.455999</v>
+        <v>8370000000</v>
       </c>
       <c r="Q3" s="18" t="n">
-        <v>10545492268.55424</v>
+        <v>9156000000</v>
       </c>
     </row>
     <row r="4">
@@ -1766,49 +1796,49 @@
           <t>Accounts Receivable</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n"/>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="17" t="n">
+      <c r="B4" s="17" t="n"/>
+      <c r="C4" s="17" t="n"/>
+      <c r="D4" s="16" t="n">
         <v>1238100000</v>
       </c>
-      <c r="E4" s="17" t="n">
+      <c r="E4" s="16" t="n">
         <v>1278100000</v>
       </c>
-      <c r="F4" s="17" t="n">
+      <c r="F4" s="16" t="n">
+        <v>2142500000</v>
+      </c>
+      <c r="G4" s="16" t="n">
         <v>1443600000</v>
       </c>
-      <c r="G4" s="17" t="n">
-        <v>2142500000</v>
-      </c>
-      <c r="H4" s="17" t="n">
+      <c r="H4" s="16" t="n">
         <v>1715400000</v>
       </c>
-      <c r="I4" s="17" t="n">
+      <c r="I4" s="16" t="n">
         <v>1950000000</v>
       </c>
-      <c r="J4" s="17" t="n">
+      <c r="J4" s="16" t="n">
+        <v>1343000000</v>
+      </c>
+      <c r="K4" s="16" t="n">
         <v>2965000000</v>
       </c>
-      <c r="K4" s="17" t="n">
-        <v>1343000000</v>
-      </c>
-      <c r="L4" s="17" t="n">
+      <c r="L4" s="16" t="n">
         <v>2965000000</v>
       </c>
-      <c r="M4" s="17" t="n">
+      <c r="M4" s="16" t="n">
         <v>2116000000</v>
       </c>
       <c r="N4" s="18" t="n">
-        <v>2200640000</v>
+        <v>0</v>
       </c>
       <c r="O4" s="18" t="n">
-        <v>2288665600</v>
+        <v>0</v>
       </c>
       <c r="P4" s="18" t="n">
-        <v>2380212224</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="18" t="n">
-        <v>2475420712.96</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1817,18 +1847,18 @@
           <t>Inventory</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n"/>
-      <c r="C5" s="16" t="n"/>
-      <c r="D5" s="16" t="n"/>
-      <c r="E5" s="16" t="n"/>
-      <c r="F5" s="16" t="n"/>
-      <c r="G5" s="16" t="n"/>
-      <c r="H5" s="16" t="n"/>
-      <c r="I5" s="16" t="n"/>
-      <c r="J5" s="16" t="n"/>
-      <c r="K5" s="16" t="n"/>
-      <c r="L5" s="16" t="n"/>
-      <c r="M5" s="16" t="n"/>
+      <c r="B5" s="17" t="n"/>
+      <c r="C5" s="17" t="n"/>
+      <c r="D5" s="17" t="n"/>
+      <c r="E5" s="17" t="n"/>
+      <c r="F5" s="17" t="n"/>
+      <c r="G5" s="17" t="n"/>
+      <c r="H5" s="17" t="n"/>
+      <c r="I5" s="17" t="n"/>
+      <c r="J5" s="17" t="n"/>
+      <c r="K5" s="17" t="n"/>
+      <c r="L5" s="17" t="n"/>
+      <c r="M5" s="17" t="n"/>
       <c r="N5" s="18" t="n">
         <v>0</v>
       </c>
@@ -1848,49 +1878,49 @@
           <t>TOTAL ASSETS</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n"/>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="17" t="n">
+      <c r="B6" s="17" t="n"/>
+      <c r="C6" s="17" t="n"/>
+      <c r="D6" s="16" t="n">
         <v>12543800000</v>
       </c>
-      <c r="E6" s="17" t="n">
+      <c r="E6" s="16" t="n">
         <v>13163400000</v>
       </c>
-      <c r="F6" s="17" t="n">
+      <c r="F6" s="16" t="n">
+        <v>12253600000</v>
+      </c>
+      <c r="G6" s="16" t="n">
         <v>14170500000</v>
       </c>
-      <c r="G6" s="17" t="n">
-        <v>12253600000</v>
-      </c>
-      <c r="H6" s="17" t="n">
+      <c r="H6" s="16" t="n">
         <v>17930800000</v>
       </c>
-      <c r="I6" s="17" t="n">
+      <c r="I6" s="16" t="n">
         <v>22002800000</v>
       </c>
-      <c r="J6" s="17" t="n">
+      <c r="J6" s="16" t="n">
+        <v>23536000000</v>
+      </c>
+      <c r="K6" s="16" t="n">
         <v>23576000000</v>
       </c>
-      <c r="K6" s="17" t="n">
-        <v>23536000000</v>
-      </c>
-      <c r="L6" s="17" t="n">
+      <c r="L6" s="16" t="n">
         <v>23576000000</v>
       </c>
-      <c r="M6" s="17" t="n">
+      <c r="M6" s="16" t="n">
         <v>24979000000</v>
       </c>
       <c r="N6" s="18" t="n">
-        <v>26009412000</v>
+        <v>25332000000</v>
       </c>
       <c r="O6" s="18" t="n">
-        <v>27524291680</v>
+        <v>25947000000</v>
       </c>
       <c r="P6" s="18" t="n">
-        <v>29454367507.2</v>
+        <v>26562000000</v>
       </c>
       <c r="Q6" s="18" t="n">
-        <v>31745327135.488</v>
+        <v>27177000000</v>
       </c>
     </row>
     <row r="8">
@@ -1906,49 +1936,49 @@
           <t>Accounts Payable</t>
         </is>
       </c>
-      <c r="B9" s="16" t="n"/>
-      <c r="C9" s="16" t="n"/>
-      <c r="D9" s="17" t="n">
+      <c r="B9" s="17" t="n"/>
+      <c r="C9" s="17" t="n"/>
+      <c r="D9" s="16" t="n">
         <v>125900000</v>
       </c>
-      <c r="E9" s="17" t="n">
+      <c r="E9" s="16" t="n">
         <v>128300000</v>
       </c>
-      <c r="F9" s="17" t="n">
+      <c r="F9" s="16" t="n">
+        <v>128000000</v>
+      </c>
+      <c r="G9" s="16" t="n">
         <v>91600000</v>
       </c>
-      <c r="G9" s="17" t="n">
-        <v>128000000</v>
-      </c>
-      <c r="H9" s="17" t="n">
+      <c r="H9" s="16" t="n">
         <v>108900000</v>
       </c>
-      <c r="I9" s="17" t="n">
+      <c r="I9" s="16" t="n">
         <v>234800000</v>
       </c>
-      <c r="J9" s="17" t="n">
+      <c r="J9" s="16" t="n">
+        <v>223000000</v>
+      </c>
+      <c r="K9" s="16" t="n">
         <v>232000000</v>
       </c>
-      <c r="K9" s="17" t="n">
-        <v>223000000</v>
-      </c>
-      <c r="L9" s="17" t="n">
+      <c r="L9" s="16" t="n">
         <v>232000000</v>
       </c>
-      <c r="M9" s="17" t="n">
+      <c r="M9" s="16" t="n">
         <v>262000000</v>
       </c>
       <c r="N9" s="18" t="n">
-        <v>272479999.9999999</v>
+        <v>0</v>
       </c>
       <c r="O9" s="18" t="n">
-        <v>283379199.9999999</v>
+        <v>0</v>
       </c>
       <c r="P9" s="18" t="n">
-        <v>294714367.9999999</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="18" t="n">
-        <v>306502942.72</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1957,36 +1987,36 @@
           <t>Deferred Revenue</t>
         </is>
       </c>
-      <c r="B10" s="16" t="n"/>
-      <c r="C10" s="16" t="n"/>
-      <c r="D10" s="17" t="n">
+      <c r="B10" s="17" t="n"/>
+      <c r="C10" s="17" t="n"/>
+      <c r="D10" s="16" t="n">
         <v>3741300000</v>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="E10" s="16" t="n">
         <v>3942500000</v>
       </c>
-      <c r="F10" s="17" t="n">
+      <c r="F10" s="16" t="n">
+        <v>3641200000</v>
+      </c>
+      <c r="G10" s="16" t="n">
         <v>4146700000</v>
       </c>
-      <c r="G10" s="17" t="n">
-        <v>3641200000</v>
-      </c>
-      <c r="H10" s="17" t="n">
+      <c r="H10" s="16" t="n">
         <v>5014900000</v>
       </c>
-      <c r="I10" s="17" t="n">
+      <c r="I10" s="16" t="n">
         <v>5756800000</v>
       </c>
-      <c r="J10" s="17" t="n">
+      <c r="J10" s="16" t="n">
+        <v>6132000000</v>
+      </c>
+      <c r="K10" s="16" t="n">
         <v>6302000000</v>
       </c>
-      <c r="K10" s="17" t="n">
-        <v>6132000000</v>
-      </c>
-      <c r="L10" s="17" t="n">
+      <c r="L10" s="16" t="n">
         <v>6302000000</v>
       </c>
-      <c r="M10" s="17" t="n">
+      <c r="M10" s="16" t="n">
         <v>6248000000</v>
       </c>
       <c r="N10" s="18" t="n">
@@ -2008,49 +2038,49 @@
           <t>TOTAL LIABILITIES</t>
         </is>
       </c>
-      <c r="B11" s="16" t="n"/>
-      <c r="C11" s="16" t="n"/>
-      <c r="D11" s="17" t="n">
+      <c r="B11" s="17" t="n"/>
+      <c r="C11" s="17" t="n"/>
+      <c r="D11" s="16" t="n">
         <v>12035800000</v>
       </c>
-      <c r="E11" s="17" t="n">
+      <c r="E11" s="16" t="n">
         <v>12434400000</v>
       </c>
-      <c r="F11" s="17" t="n">
+      <c r="F11" s="16" t="n">
+        <v>12043600000</v>
+      </c>
+      <c r="G11" s="16" t="n">
         <v>12938100000</v>
       </c>
-      <c r="G11" s="17" t="n">
-        <v>12043600000</v>
-      </c>
-      <c r="H11" s="17" t="n">
+      <c r="H11" s="16" t="n">
         <v>13463000000</v>
       </c>
-      <c r="I11" s="17" t="n">
+      <c r="I11" s="16" t="n">
         <v>14772300000</v>
       </c>
-      <c r="J11" s="17" t="n">
+      <c r="J11" s="16" t="n">
+        <v>14871000000</v>
+      </c>
+      <c r="K11" s="16" t="n">
         <v>15752000000</v>
       </c>
-      <c r="K11" s="17" t="n">
-        <v>14871000000</v>
-      </c>
-      <c r="L11" s="17" t="n">
+      <c r="L11" s="16" t="n">
         <v>15752000000</v>
       </c>
-      <c r="M11" s="17" t="n">
+      <c r="M11" s="16" t="n">
         <v>15586000000</v>
       </c>
       <c r="N11" s="18" t="n">
-        <v>15596480000</v>
+        <v>15324000000</v>
       </c>
       <c r="O11" s="18" t="n">
-        <v>15607379200</v>
+        <v>15324000000</v>
       </c>
       <c r="P11" s="18" t="n">
-        <v>15618714368</v>
+        <v>15324000000</v>
       </c>
       <c r="Q11" s="18" t="n">
-        <v>15630502942.72</v>
+        <v>15324000000</v>
       </c>
     </row>
     <row r="13">
@@ -2066,49 +2096,49 @@
           <t>Total Equity</t>
         </is>
       </c>
-      <c r="B14" s="16" t="n"/>
-      <c r="C14" s="16" t="n"/>
-      <c r="D14" s="17" t="n">
+      <c r="B14" s="17" t="n"/>
+      <c r="C14" s="17" t="n"/>
+      <c r="D14" s="16" t="n">
         <v>508000000</v>
       </c>
-      <c r="E14" s="17" t="n">
+      <c r="E14" s="16" t="n">
         <v>729000000</v>
       </c>
-      <c r="F14" s="17" t="n">
+      <c r="F14" s="16" t="n">
+        <v>210000000</v>
+      </c>
+      <c r="G14" s="16" t="n">
         <v>1232400000</v>
       </c>
-      <c r="G14" s="17" t="n">
-        <v>210000000</v>
-      </c>
-      <c r="H14" s="17" t="n">
+      <c r="H14" s="16" t="n">
         <v>4467800000</v>
       </c>
-      <c r="I14" s="17" t="n">
+      <c r="I14" s="16" t="n">
         <v>7230500000</v>
       </c>
-      <c r="J14" s="17" t="n">
+      <c r="J14" s="16" t="n">
+        <v>8665000000</v>
+      </c>
+      <c r="K14" s="16" t="n">
         <v>7824000000</v>
       </c>
-      <c r="K14" s="17" t="n">
-        <v>8665000000</v>
-      </c>
-      <c r="L14" s="17" t="n">
+      <c r="L14" s="16" t="n">
         <v>7824000000</v>
       </c>
-      <c r="M14" s="17" t="n">
+      <c r="M14" s="16" t="n">
         <v>9393000000</v>
       </c>
       <c r="N14" s="18" t="n">
-        <v>10412932000</v>
+        <v>10008000000</v>
       </c>
       <c r="O14" s="18" t="n">
-        <v>11916912480</v>
+        <v>10623000000</v>
       </c>
       <c r="P14" s="18" t="n">
-        <v>13835653139.2</v>
+        <v>11238000000</v>
       </c>
       <c r="Q14" s="18" t="n">
-        <v>16114824192.768</v>
+        <v>11853000000</v>
       </c>
     </row>
     <row r="16">
@@ -2124,10 +2154,10 @@
         <v>0</v>
       </c>
       <c r="P16" s="23" t="n">
-        <v>-3.814697265625e-06</v>
+        <v>0</v>
       </c>
       <c r="Q16" s="23" t="n">
-        <v>-3.814697265625e-06</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2263,37 +2293,41 @@
           <t>Net Income</t>
         </is>
       </c>
-      <c r="B3" s="16" t="n"/>
-      <c r="C3" s="16" t="n"/>
-      <c r="D3" s="17" t="n">
+      <c r="B3" s="16" t="n">
+        <v>880100000</v>
+      </c>
+      <c r="C3" s="16" t="n">
+        <v>2219900000</v>
+      </c>
+      <c r="D3" s="16" t="n">
+        <v>351000000</v>
+      </c>
+      <c r="E3" s="16" t="n">
         <v>334000000</v>
       </c>
-      <c r="E3" s="16" t="n"/>
-      <c r="F3" s="16" t="n"/>
-      <c r="G3" s="17" t="n">
-        <v>351000000</v>
-      </c>
-      <c r="H3" s="16" t="n"/>
-      <c r="I3" s="16" t="n"/>
-      <c r="J3" s="16" t="n"/>
-      <c r="K3" s="17" t="n">
+      <c r="F3" s="17" t="n"/>
+      <c r="G3" s="17" t="n"/>
+      <c r="H3" s="17" t="n"/>
+      <c r="I3" s="16" t="n">
         <v>766000000</v>
       </c>
-      <c r="L3" s="16" t="n"/>
-      <c r="M3" s="17" t="n">
+      <c r="J3" s="17" t="n"/>
+      <c r="K3" s="17" t="n"/>
+      <c r="L3" s="16" t="n">
         <v>618000000</v>
       </c>
+      <c r="M3" s="17" t="n"/>
       <c r="N3" s="18" t="n">
-        <v>1019932000</v>
+        <v>0</v>
       </c>
       <c r="O3" s="18" t="n">
-        <v>1503980480</v>
+        <v>0</v>
       </c>
       <c r="P3" s="18" t="n">
-        <v>1918740659.2</v>
+        <v>0</v>
       </c>
       <c r="Q3" s="18" t="n">
-        <v>2279171053.568</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -2302,39 +2336,37 @@
           <t>Depreciation &amp; Amort</t>
         </is>
       </c>
-      <c r="B4" s="17" t="n">
-        <v>207200000</v>
-      </c>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="17" t="n">
+      <c r="B4" s="17" t="n"/>
+      <c r="C4" s="17" t="n"/>
+      <c r="D4" s="17" t="n"/>
+      <c r="E4" s="17" t="n"/>
+      <c r="F4" s="16" t="n">
+        <v>84000000</v>
+      </c>
+      <c r="G4" s="16" t="n">
         <v>89000000</v>
       </c>
-      <c r="E4" s="16" t="n"/>
-      <c r="F4" s="16" t="n"/>
-      <c r="G4" s="17" t="n">
-        <v>84000000</v>
-      </c>
-      <c r="H4" s="16" t="n"/>
-      <c r="I4" s="17" t="n">
+      <c r="H4" s="17" t="n"/>
+      <c r="I4" s="17" t="n"/>
+      <c r="J4" s="17" t="n"/>
+      <c r="K4" s="16" t="n">
+        <v>180000000</v>
+      </c>
+      <c r="L4" s="17" t="n"/>
+      <c r="M4" s="16" t="n">
         <v>171000000</v>
       </c>
-      <c r="J4" s="16" t="n"/>
-      <c r="K4" s="17" t="n">
-        <v>180000000</v>
-      </c>
-      <c r="L4" s="16" t="n"/>
-      <c r="M4" s="16" t="n"/>
       <c r="N4" s="18" t="n">
-        <v>0</v>
+        <v>171000000</v>
       </c>
       <c r="O4" s="18" t="n">
-        <v>0</v>
+        <v>171000000</v>
       </c>
       <c r="P4" s="18" t="n">
-        <v>0</v>
+        <v>171000000</v>
       </c>
       <c r="Q4" s="18" t="n">
-        <v>0</v>
+        <v>171000000</v>
       </c>
     </row>
     <row r="5">
@@ -2343,39 +2375,37 @@
           <t>Stock-Based Comp</t>
         </is>
       </c>
-      <c r="B5" s="17" t="n">
-        <v>806500000</v>
-      </c>
-      <c r="C5" s="16" t="n"/>
-      <c r="D5" s="17" t="n">
+      <c r="B5" s="17" t="n"/>
+      <c r="C5" s="17" t="n"/>
+      <c r="D5" s="17" t="n"/>
+      <c r="E5" s="17" t="n"/>
+      <c r="F5" s="16" t="n">
+        <v>295000000</v>
+      </c>
+      <c r="G5" s="16" t="n">
         <v>370000000</v>
       </c>
-      <c r="E5" s="16" t="n"/>
-      <c r="F5" s="16" t="n"/>
-      <c r="G5" s="17" t="n">
-        <v>295000000</v>
-      </c>
-      <c r="H5" s="16" t="n"/>
-      <c r="I5" s="17" t="n">
+      <c r="H5" s="17" t="n"/>
+      <c r="I5" s="17" t="n"/>
+      <c r="J5" s="17" t="n"/>
+      <c r="K5" s="16" t="n">
+        <v>671000000</v>
+      </c>
+      <c r="L5" s="17" t="n"/>
+      <c r="M5" s="16" t="n">
         <v>615000000</v>
       </c>
-      <c r="J5" s="16" t="n"/>
-      <c r="K5" s="17" t="n">
-        <v>671000000</v>
-      </c>
-      <c r="L5" s="16" t="n"/>
-      <c r="M5" s="16" t="n"/>
       <c r="N5" s="18" t="n">
-        <v>0</v>
+        <v>615000000</v>
       </c>
       <c r="O5" s="18" t="n">
-        <v>0</v>
+        <v>615000000</v>
       </c>
       <c r="P5" s="18" t="n">
-        <v>0</v>
+        <v>615000000</v>
       </c>
       <c r="Q5" s="18" t="n">
-        <v>0</v>
+        <v>615000000</v>
       </c>
     </row>
     <row r="6">
@@ -2384,47 +2414,45 @@
           <t>Δ Accounts Receivable (−increase)</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n"/>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="16" t="n"/>
-      <c r="E6" s="17" t="n">
+      <c r="B6" s="17" t="n"/>
+      <c r="C6" s="17" t="n"/>
+      <c r="D6" s="17" t="n"/>
+      <c r="E6" s="16" t="n">
         <v>-40000000</v>
       </c>
-      <c r="F6" s="17" t="n">
-        <v>-165500000</v>
-      </c>
-      <c r="G6" s="17" t="n">
-        <v>-698900000</v>
-      </c>
-      <c r="H6" s="17" t="n">
-        <v>427100000</v>
-      </c>
-      <c r="I6" s="17" t="n">
+      <c r="F6" s="16" t="n">
+        <v>-864400000</v>
+      </c>
+      <c r="G6" s="16" t="n">
+        <v>698900000</v>
+      </c>
+      <c r="H6" s="16" t="n">
+        <v>-271800000</v>
+      </c>
+      <c r="I6" s="16" t="n">
         <v>-234600000</v>
       </c>
-      <c r="J6" s="17" t="n">
-        <v>-1015000000</v>
-      </c>
-      <c r="K6" s="17" t="n">
-        <v>1622000000</v>
-      </c>
-      <c r="L6" s="17" t="n">
+      <c r="J6" s="16" t="n">
+        <v>607000000</v>
+      </c>
+      <c r="K6" s="16" t="n">
         <v>-1622000000</v>
       </c>
-      <c r="M6" s="17" t="n">
+      <c r="L6" s="17" t="n"/>
+      <c r="M6" s="16" t="n">
         <v>849000000</v>
       </c>
       <c r="N6" s="18" t="n">
-        <v>-84640000</v>
+        <v>2116000000</v>
       </c>
       <c r="O6" s="18" t="n">
-        <v>-88025600</v>
+        <v>-0</v>
       </c>
       <c r="P6" s="18" t="n">
-        <v>-91546624</v>
+        <v>-0</v>
       </c>
       <c r="Q6" s="18" t="n">
-        <v>-95208488.96000004</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="7">
@@ -2433,18 +2461,18 @@
           <t>Δ Inventory (−increase)</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n"/>
-      <c r="C7" s="16" t="n"/>
-      <c r="D7" s="16" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="16" t="n"/>
-      <c r="G7" s="16" t="n"/>
-      <c r="H7" s="16" t="n"/>
-      <c r="I7" s="16" t="n"/>
-      <c r="J7" s="16" t="n"/>
-      <c r="K7" s="16" t="n"/>
-      <c r="L7" s="16" t="n"/>
-      <c r="M7" s="16" t="n"/>
+      <c r="B7" s="17" t="n"/>
+      <c r="C7" s="17" t="n"/>
+      <c r="D7" s="17" t="n"/>
+      <c r="E7" s="17" t="n"/>
+      <c r="F7" s="17" t="n"/>
+      <c r="G7" s="17" t="n"/>
+      <c r="H7" s="17" t="n"/>
+      <c r="I7" s="17" t="n"/>
+      <c r="J7" s="17" t="n"/>
+      <c r="K7" s="17" t="n"/>
+      <c r="L7" s="17" t="n"/>
+      <c r="M7" s="17" t="n"/>
       <c r="N7" s="18" t="n">
         <v>-0</v>
       </c>
@@ -2464,47 +2492,45 @@
           <t>Δ Accounts Payable (+increase)</t>
         </is>
       </c>
-      <c r="B8" s="16" t="n"/>
-      <c r="C8" s="16" t="n"/>
-      <c r="D8" s="16" t="n"/>
-      <c r="E8" s="17" t="n">
+      <c r="B8" s="17" t="n"/>
+      <c r="C8" s="17" t="n"/>
+      <c r="D8" s="17" t="n"/>
+      <c r="E8" s="16" t="n">
         <v>2400000</v>
       </c>
-      <c r="F8" s="17" t="n">
-        <v>-36700000</v>
-      </c>
-      <c r="G8" s="17" t="n">
-        <v>36400000</v>
-      </c>
-      <c r="H8" s="17" t="n">
-        <v>-19100000</v>
-      </c>
-      <c r="I8" s="17" t="n">
+      <c r="F8" s="16" t="n">
+        <v>-300000</v>
+      </c>
+      <c r="G8" s="16" t="n">
+        <v>-36400000</v>
+      </c>
+      <c r="H8" s="16" t="n">
+        <v>17300000</v>
+      </c>
+      <c r="I8" s="16" t="n">
         <v>125900000</v>
       </c>
-      <c r="J8" s="17" t="n">
-        <v>-2800000</v>
-      </c>
-      <c r="K8" s="17" t="n">
-        <v>-9000000</v>
-      </c>
-      <c r="L8" s="17" t="n">
+      <c r="J8" s="16" t="n">
+        <v>-11800000</v>
+      </c>
+      <c r="K8" s="16" t="n">
         <v>9000000</v>
       </c>
-      <c r="M8" s="17" t="n">
+      <c r="L8" s="17" t="n"/>
+      <c r="M8" s="16" t="n">
         <v>30000000</v>
       </c>
       <c r="N8" s="18" t="n">
-        <v>10479999.99999994</v>
+        <v>-262000000</v>
       </c>
       <c r="O8" s="18" t="n">
-        <v>10899200</v>
+        <v>0</v>
       </c>
       <c r="P8" s="18" t="n">
-        <v>11335168</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="18" t="n">
-        <v>11788574.72000003</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -2513,39 +2539,37 @@
           <t>OPERATING CASH FLOW</t>
         </is>
       </c>
-      <c r="B9" s="17" t="n">
-        <v>2744900000</v>
-      </c>
-      <c r="C9" s="16" t="n"/>
-      <c r="D9" s="17" t="n">
+      <c r="B9" s="17" t="n"/>
+      <c r="C9" s="17" t="n"/>
+      <c r="D9" s="17" t="n"/>
+      <c r="E9" s="17" t="n"/>
+      <c r="F9" s="16" t="n">
+        <v>1510000000</v>
+      </c>
+      <c r="G9" s="16" t="n">
         <v>1771000000</v>
       </c>
-      <c r="E9" s="16" t="n"/>
-      <c r="F9" s="16" t="n"/>
-      <c r="G9" s="17" t="n">
-        <v>1510000000</v>
-      </c>
-      <c r="H9" s="16" t="n"/>
-      <c r="I9" s="17" t="n">
+      <c r="H9" s="17" t="n"/>
+      <c r="I9" s="17" t="n"/>
+      <c r="J9" s="17" t="n"/>
+      <c r="K9" s="16" t="n">
+        <v>2325000000</v>
+      </c>
+      <c r="L9" s="17" t="n"/>
+      <c r="M9" s="16" t="n">
         <v>2067000000</v>
       </c>
-      <c r="J9" s="16" t="n"/>
-      <c r="K9" s="17" t="n">
-        <v>2325000000</v>
-      </c>
-      <c r="L9" s="16" t="n"/>
-      <c r="M9" s="16" t="n"/>
       <c r="N9" s="18" t="n">
-        <v>945772000</v>
+        <v>2640000000</v>
       </c>
       <c r="O9" s="18" t="n">
-        <v>1426854080</v>
+        <v>786000000</v>
       </c>
       <c r="P9" s="18" t="n">
-        <v>1838529203.2</v>
+        <v>786000000</v>
       </c>
       <c r="Q9" s="18" t="n">
-        <v>2195751139.328</v>
+        <v>786000000</v>
       </c>
     </row>
     <row r="11">
@@ -2561,29 +2585,29 @@
           <t>Capital Expenditures (−)</t>
         </is>
       </c>
-      <c r="B12" s="16" t="n"/>
-      <c r="C12" s="16" t="n"/>
-      <c r="D12" s="16" t="n"/>
-      <c r="E12" s="16" t="n"/>
-      <c r="F12" s="16" t="n"/>
-      <c r="G12" s="16" t="n"/>
-      <c r="H12" s="16" t="n"/>
-      <c r="I12" s="16" t="n"/>
-      <c r="J12" s="16" t="n"/>
-      <c r="K12" s="16" t="n"/>
-      <c r="L12" s="16" t="n"/>
-      <c r="M12" s="16" t="n"/>
+      <c r="B12" s="17" t="n"/>
+      <c r="C12" s="17" t="n"/>
+      <c r="D12" s="17" t="n"/>
+      <c r="E12" s="17" t="n"/>
+      <c r="F12" s="17" t="n"/>
+      <c r="G12" s="17" t="n"/>
+      <c r="H12" s="17" t="n"/>
+      <c r="I12" s="17" t="n"/>
+      <c r="J12" s="17" t="n"/>
+      <c r="K12" s="17" t="n"/>
+      <c r="L12" s="17" t="n"/>
+      <c r="M12" s="17" t="n"/>
       <c r="N12" s="18" t="n">
-        <v>4571840</v>
+        <v>0</v>
       </c>
       <c r="O12" s="18" t="n">
-        <v>4754713.600000001</v>
+        <v>0</v>
       </c>
       <c r="P12" s="18" t="n">
-        <v>4944902.144</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="18" t="n">
-        <v>5142698.22976</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -2592,39 +2616,37 @@
           <t>INVESTING CASH FLOW</t>
         </is>
       </c>
-      <c r="B13" s="17" t="n">
-        <v>-1341400000</v>
-      </c>
-      <c r="C13" s="16" t="n"/>
-      <c r="D13" s="17" t="n">
+      <c r="B13" s="17" t="n"/>
+      <c r="C13" s="17" t="n"/>
+      <c r="D13" s="17" t="n"/>
+      <c r="E13" s="17" t="n"/>
+      <c r="F13" s="16" t="n">
+        <v>-544000000</v>
+      </c>
+      <c r="G13" s="16" t="n">
         <v>-983000000</v>
       </c>
-      <c r="E13" s="16" t="n"/>
-      <c r="F13" s="16" t="n"/>
-      <c r="G13" s="17" t="n">
-        <v>-544000000</v>
-      </c>
-      <c r="H13" s="16" t="n"/>
-      <c r="I13" s="17" t="n">
+      <c r="H13" s="17" t="n"/>
+      <c r="I13" s="17" t="n"/>
+      <c r="J13" s="17" t="n"/>
+      <c r="K13" s="16" t="n">
+        <v>-332000000</v>
+      </c>
+      <c r="L13" s="17" t="n"/>
+      <c r="M13" s="16" t="n">
         <v>-925000000</v>
       </c>
-      <c r="J13" s="16" t="n"/>
-      <c r="K13" s="17" t="n">
-        <v>-332000000</v>
-      </c>
-      <c r="L13" s="16" t="n"/>
-      <c r="M13" s="16" t="n"/>
       <c r="N13" s="18" t="n">
-        <v>-4571840</v>
+        <v>-0</v>
       </c>
       <c r="O13" s="18" t="n">
-        <v>-4754713.600000001</v>
+        <v>-0</v>
       </c>
       <c r="P13" s="18" t="n">
-        <v>-4944902.144</v>
+        <v>-0</v>
       </c>
       <c r="Q13" s="18" t="n">
-        <v>-5142698.22976</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="15">
@@ -2640,20 +2662,18 @@
           <t>Stock Buybacks (−)</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
-        <v>566700000</v>
-      </c>
-      <c r="C16" s="16" t="n"/>
-      <c r="D16" s="16" t="n"/>
-      <c r="E16" s="16" t="n"/>
-      <c r="F16" s="16" t="n"/>
-      <c r="G16" s="16" t="n"/>
-      <c r="H16" s="16" t="n"/>
-      <c r="I16" s="16" t="n"/>
-      <c r="J16" s="16" t="n"/>
-      <c r="K16" s="16" t="n"/>
-      <c r="L16" s="16" t="n"/>
-      <c r="M16" s="16" t="n"/>
+      <c r="B16" s="17" t="n"/>
+      <c r="C16" s="17" t="n"/>
+      <c r="D16" s="17" t="n"/>
+      <c r="E16" s="17" t="n"/>
+      <c r="F16" s="17" t="n"/>
+      <c r="G16" s="17" t="n"/>
+      <c r="H16" s="17" t="n"/>
+      <c r="I16" s="17" t="n"/>
+      <c r="J16" s="17" t="n"/>
+      <c r="K16" s="17" t="n"/>
+      <c r="L16" s="17" t="n"/>
+      <c r="M16" s="17" t="n"/>
       <c r="N16" s="18" t="n">
         <v>0</v>
       </c>
@@ -2673,28 +2693,26 @@
           <t>FINANCING CASH FLOW</t>
         </is>
       </c>
-      <c r="B17" s="17" t="n">
-        <v>-1163800000</v>
-      </c>
-      <c r="C17" s="16" t="n"/>
-      <c r="D17" s="17" t="n">
+      <c r="B17" s="17" t="n"/>
+      <c r="C17" s="17" t="n"/>
+      <c r="D17" s="17" t="n"/>
+      <c r="E17" s="17" t="n"/>
+      <c r="F17" s="16" t="n">
+        <v>-220000000</v>
+      </c>
+      <c r="G17" s="16" t="n">
         <v>8000000</v>
       </c>
-      <c r="E17" s="16" t="n"/>
-      <c r="F17" s="16" t="n"/>
-      <c r="G17" s="17" t="n">
-        <v>-220000000</v>
-      </c>
-      <c r="H17" s="16" t="n"/>
-      <c r="I17" s="17" t="n">
+      <c r="H17" s="17" t="n"/>
+      <c r="I17" s="17" t="n"/>
+      <c r="J17" s="17" t="n"/>
+      <c r="K17" s="16" t="n">
+        <v>-106000000</v>
+      </c>
+      <c r="L17" s="17" t="n"/>
+      <c r="M17" s="16" t="n">
         <v>-452000000</v>
       </c>
-      <c r="J17" s="16" t="n"/>
-      <c r="K17" s="17" t="n">
-        <v>-106000000</v>
-      </c>
-      <c r="L17" s="16" t="n"/>
-      <c r="M17" s="16" t="n"/>
       <c r="N17" s="18" t="n">
         <v>-0</v>
       </c>
@@ -2714,29 +2732,29 @@
           <t>Net Change in Cash</t>
         </is>
       </c>
-      <c r="B19" s="16" t="n"/>
-      <c r="C19" s="16" t="n"/>
-      <c r="D19" s="16" t="n"/>
-      <c r="E19" s="16" t="n"/>
-      <c r="F19" s="16" t="n"/>
-      <c r="G19" s="16" t="n"/>
-      <c r="H19" s="16" t="n"/>
-      <c r="I19" s="16" t="n"/>
-      <c r="J19" s="16" t="n"/>
-      <c r="K19" s="16" t="n"/>
-      <c r="L19" s="16" t="n"/>
-      <c r="M19" s="16" t="n"/>
+      <c r="B19" s="17" t="n"/>
+      <c r="C19" s="17" t="n"/>
+      <c r="D19" s="17" t="n"/>
+      <c r="E19" s="17" t="n"/>
+      <c r="F19" s="17" t="n"/>
+      <c r="G19" s="17" t="n"/>
+      <c r="H19" s="17" t="n"/>
+      <c r="I19" s="17" t="n"/>
+      <c r="J19" s="17" t="n"/>
+      <c r="K19" s="17" t="n"/>
+      <c r="L19" s="17" t="n"/>
+      <c r="M19" s="17" t="n"/>
       <c r="N19" s="18" t="n">
-        <v>941200160</v>
+        <v>2640000000</v>
       </c>
       <c r="O19" s="18" t="n">
-        <v>1422099366.4</v>
+        <v>786000000</v>
       </c>
       <c r="P19" s="18" t="n">
-        <v>1833584301.056</v>
+        <v>786000000</v>
       </c>
       <c r="Q19" s="18" t="n">
-        <v>2190608441.09824</v>
+        <v>786000000</v>
       </c>
     </row>
     <row r="20">
@@ -2745,29 +2763,29 @@
           <t>Ending Cash (= BS Cash)</t>
         </is>
       </c>
-      <c r="B20" s="16" t="n"/>
-      <c r="C20" s="16" t="n"/>
-      <c r="D20" s="16" t="n"/>
-      <c r="E20" s="16" t="n"/>
-      <c r="F20" s="16" t="n"/>
-      <c r="G20" s="16" t="n"/>
-      <c r="H20" s="16" t="n"/>
-      <c r="I20" s="16" t="n"/>
-      <c r="J20" s="16" t="n"/>
-      <c r="K20" s="16" t="n"/>
-      <c r="L20" s="16" t="n"/>
-      <c r="M20" s="16" t="n"/>
+      <c r="B20" s="17" t="n"/>
+      <c r="C20" s="17" t="n"/>
+      <c r="D20" s="17" t="n"/>
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="17" t="n"/>
+      <c r="G20" s="17" t="n"/>
+      <c r="H20" s="17" t="n"/>
+      <c r="I20" s="17" t="n"/>
+      <c r="J20" s="17" t="n"/>
+      <c r="K20" s="17" t="n"/>
+      <c r="L20" s="17" t="n"/>
+      <c r="M20" s="17" t="n"/>
       <c r="N20" s="18" t="n">
-        <v>5099200160</v>
+        <v>6798000000</v>
       </c>
       <c r="O20" s="18" t="n">
-        <v>6521299526.4</v>
+        <v>7584000000</v>
       </c>
       <c r="P20" s="18" t="n">
-        <v>8354883827.455999</v>
+        <v>8370000000</v>
       </c>
       <c r="Q20" s="18" t="n">
-        <v>10545492268.55424</v>
+        <v>9156000000</v>
       </c>
     </row>
   </sheetData>
@@ -3037,37 +3055,41 @@
           <t>Revenue ($)</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n"/>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="17" t="n">
+      <c r="B4" s="16" t="n">
+        <v>6685200000</v>
+      </c>
+      <c r="C4" s="16" t="n">
+        <v>5838000000</v>
+      </c>
+      <c r="D4" s="16" t="n">
+        <v>2139000000</v>
+      </c>
+      <c r="E4" s="16" t="n">
         <v>2474000000</v>
       </c>
-      <c r="E4" s="16" t="n"/>
-      <c r="F4" s="16" t="n"/>
-      <c r="G4" s="17" t="n">
-        <v>2139000000</v>
-      </c>
-      <c r="H4" s="16" t="n"/>
-      <c r="I4" s="16" t="n"/>
-      <c r="J4" s="16" t="n"/>
-      <c r="K4" s="17" t="n">
+      <c r="F4" s="17" t="n"/>
+      <c r="G4" s="17" t="n"/>
+      <c r="H4" s="17" t="n"/>
+      <c r="I4" s="16" t="n">
         <v>5068000000</v>
       </c>
-      <c r="L4" s="16" t="n"/>
-      <c r="M4" s="17" t="n">
+      <c r="J4" s="17" t="n"/>
+      <c r="K4" s="17" t="n"/>
+      <c r="L4" s="16" t="n">
         <v>4396000000</v>
       </c>
+      <c r="M4" s="17" t="n"/>
       <c r="N4" s="18" t="n">
-        <v>4571840000</v>
+        <v>0</v>
       </c>
       <c r="O4" s="18" t="n">
-        <v>4754713600</v>
+        <v>0</v>
       </c>
       <c r="P4" s="18" t="n">
-        <v>4944902144</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="18" t="n">
-        <v>5142698229.76</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -3076,37 +3098,41 @@
           <t>Operating Income ($)</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n"/>
-      <c r="C5" s="16" t="n"/>
-      <c r="D5" s="17" t="n">
+      <c r="B5" s="16" t="n">
+        <v>745700000</v>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>445500000</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>286000000</v>
+      </c>
+      <c r="E5" s="16" t="n">
         <v>309000000</v>
       </c>
-      <c r="E5" s="16" t="n"/>
-      <c r="F5" s="16" t="n"/>
-      <c r="G5" s="17" t="n">
-        <v>286000000</v>
-      </c>
-      <c r="H5" s="16" t="n"/>
-      <c r="I5" s="16" t="n"/>
-      <c r="J5" s="16" t="n"/>
-      <c r="K5" s="17" t="n">
+      <c r="F5" s="17" t="n"/>
+      <c r="G5" s="17" t="n"/>
+      <c r="H5" s="17" t="n"/>
+      <c r="I5" s="16" t="n">
         <v>706000000</v>
       </c>
-      <c r="L5" s="16" t="n"/>
-      <c r="M5" s="17" t="n">
+      <c r="J5" s="17" t="n"/>
+      <c r="K5" s="17" t="n"/>
+      <c r="L5" s="16" t="n">
         <v>527000000</v>
       </c>
+      <c r="M5" s="17" t="n"/>
       <c r="N5" s="18" t="n">
-        <v>1199920000</v>
+        <v>0</v>
       </c>
       <c r="O5" s="18" t="n">
-        <v>1769388800</v>
+        <v>0</v>
       </c>
       <c r="P5" s="18" t="n">
-        <v>2257341952</v>
+        <v>0</v>
       </c>
       <c r="Q5" s="18" t="n">
-        <v>2681377710.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -3115,37 +3141,41 @@
           <t>Net Income ($)</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n"/>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="17" t="n">
+      <c r="B6" s="16" t="n">
+        <v>880100000</v>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>2219900000</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>351000000</v>
+      </c>
+      <c r="E6" s="16" t="n">
         <v>334000000</v>
       </c>
-      <c r="E6" s="16" t="n"/>
-      <c r="F6" s="16" t="n"/>
-      <c r="G6" s="17" t="n">
-        <v>351000000</v>
-      </c>
-      <c r="H6" s="16" t="n"/>
-      <c r="I6" s="16" t="n"/>
-      <c r="J6" s="16" t="n"/>
-      <c r="K6" s="17" t="n">
+      <c r="F6" s="17" t="n"/>
+      <c r="G6" s="17" t="n"/>
+      <c r="H6" s="17" t="n"/>
+      <c r="I6" s="16" t="n">
         <v>766000000</v>
       </c>
-      <c r="L6" s="16" t="n"/>
-      <c r="M6" s="17" t="n">
+      <c r="J6" s="17" t="n"/>
+      <c r="K6" s="17" t="n"/>
+      <c r="L6" s="16" t="n">
         <v>618000000</v>
       </c>
+      <c r="M6" s="17" t="n"/>
       <c r="N6" s="18" t="n">
-        <v>1019932000</v>
+        <v>0</v>
       </c>
       <c r="O6" s="18" t="n">
-        <v>1503980480</v>
+        <v>0</v>
       </c>
       <c r="P6" s="18" t="n">
-        <v>1918740659.2</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="18" t="n">
-        <v>2279171053.568</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -3154,39 +3184,37 @@
           <t>Operating Cash Flow ($)</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n">
-        <v>2744900000</v>
-      </c>
-      <c r="C7" s="16" t="n"/>
-      <c r="D7" s="17" t="n">
+      <c r="B7" s="17" t="n"/>
+      <c r="C7" s="17" t="n"/>
+      <c r="D7" s="17" t="n"/>
+      <c r="E7" s="17" t="n"/>
+      <c r="F7" s="16" t="n">
+        <v>1510000000</v>
+      </c>
+      <c r="G7" s="16" t="n">
         <v>1771000000</v>
       </c>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="16" t="n"/>
-      <c r="G7" s="17" t="n">
-        <v>1510000000</v>
-      </c>
-      <c r="H7" s="16" t="n"/>
-      <c r="I7" s="17" t="n">
+      <c r="H7" s="17" t="n"/>
+      <c r="I7" s="17" t="n"/>
+      <c r="J7" s="17" t="n"/>
+      <c r="K7" s="16" t="n">
+        <v>2325000000</v>
+      </c>
+      <c r="L7" s="17" t="n"/>
+      <c r="M7" s="16" t="n">
         <v>2067000000</v>
       </c>
-      <c r="J7" s="16" t="n"/>
-      <c r="K7" s="17" t="n">
-        <v>2325000000</v>
-      </c>
-      <c r="L7" s="16" t="n"/>
-      <c r="M7" s="16" t="n"/>
       <c r="N7" s="18" t="n">
-        <v>945772000</v>
+        <v>2640000000</v>
       </c>
       <c r="O7" s="18" t="n">
-        <v>1426854080</v>
+        <v>786000000</v>
       </c>
       <c r="P7" s="18" t="n">
-        <v>1838529203.2</v>
+        <v>786000000</v>
       </c>
       <c r="Q7" s="18" t="n">
-        <v>2195751139.328</v>
+        <v>786000000</v>
       </c>
     </row>
     <row r="9">
@@ -3199,7 +3227,7 @@
     <row r="10">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>Max |Modelled OCF − Reported OCF| (last 4Q): $162,000,000  ✗ FAIL (tolerance $5M)</t>
+          <t>Max |Modelled OCF − Reported OCF| (last 4Q): $649,000,000  ✗ FAIL (tolerance $5M)</t>
         </is>
       </c>
     </row>
@@ -4463,7 +4491,7 @@
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
@@ -4475,12 +4503,12 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>0001327567-23-000014</t>
+          <t>0001327567-22-000016</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000014/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000016/</t>
         </is>
       </c>
     </row>
@@ -4496,7 +4524,7 @@
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
@@ -4508,12 +4536,12 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>0001327567-22-000016</t>
+          <t>0001327567-23-000014</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000016/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000014/</t>
         </is>
       </c>
     </row>
@@ -4826,7 +4854,7 @@
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
@@ -4838,12 +4866,12 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>0001327567-23-000032</t>
+          <t>0001327567-22-000038</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000038/</t>
         </is>
       </c>
     </row>
@@ -4859,7 +4887,7 @@
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
@@ -4871,12 +4899,12 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>0001327567-22-000038</t>
+          <t>0001327567-23-000032</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000038/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
         </is>
       </c>
     </row>
@@ -4892,7 +4920,7 @@
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
@@ -4904,12 +4932,12 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>0001327567-23-000032</t>
+          <t>0001327567-22-000038</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000038/</t>
         </is>
       </c>
     </row>
@@ -4925,7 +4953,7 @@
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
@@ -4937,12 +4965,12 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>0001327567-22-000038</t>
+          <t>0001327567-23-000032</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000038/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
         </is>
       </c>
     </row>
@@ -4958,7 +4986,7 @@
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
@@ -4970,12 +4998,12 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>0001327567-23-000032</t>
+          <t>0001327567-22-000038</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000038/</t>
         </is>
       </c>
     </row>
@@ -4991,7 +5019,7 @@
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
@@ -5003,12 +5031,12 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>0001327567-22-000038</t>
+          <t>0001327567-23-000032</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000038/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
         </is>
       </c>
     </row>
@@ -5024,7 +5052,7 @@
         </is>
       </c>
       <c r="C55" s="2" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
@@ -5036,12 +5064,12 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>0001327567-22-000038</t>
+          <t>0001327567-23-000032</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000038/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
         </is>
       </c>
     </row>
@@ -5057,7 +5085,7 @@
         </is>
       </c>
       <c r="C56" s="2" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
@@ -5069,12 +5097,12 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>0001327567-23-000032</t>
+          <t>0001327567-22-000038</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000038/</t>
         </is>
       </c>
     </row>
@@ -5354,7 +5382,7 @@
         </is>
       </c>
       <c r="C65" s="2" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
@@ -5366,12 +5394,12 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>0001327567-24-000017</t>
+          <t>0001327567-23-000014</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000017/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000014/</t>
         </is>
       </c>
     </row>
@@ -5387,7 +5415,7 @@
         </is>
       </c>
       <c r="C66" s="2" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
@@ -5399,12 +5427,12 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>0001327567-23-000014</t>
+          <t>0001327567-24-000017</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000014/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000017/</t>
         </is>
       </c>
     </row>
@@ -6674,7 +6702,7 @@
         </is>
       </c>
       <c r="C105" s="2" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
@@ -6682,16 +6710,16 @@
         </is>
       </c>
       <c r="E105" s="27" t="n">
-        <v>1509600000</v>
+        <v>1510000000</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>0001327567-24-000040</t>
+          <t>0001327567-25-000035</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000035/</t>
         </is>
       </c>
     </row>
@@ -6707,7 +6735,7 @@
         </is>
       </c>
       <c r="C106" s="2" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
@@ -6715,16 +6743,16 @@
         </is>
       </c>
       <c r="E106" s="27" t="n">
-        <v>1510000000</v>
+        <v>1509600000</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>0001327567-25-000035</t>
+          <t>0001327567-24-000040</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000035/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
         </is>
       </c>
     </row>
@@ -6740,7 +6768,7 @@
         </is>
       </c>
       <c r="C107" s="2" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
@@ -6748,16 +6776,16 @@
         </is>
       </c>
       <c r="E107" s="27" t="n">
-        <v>286000000</v>
+        <v>286500000</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>0001327567-25-000035</t>
+          <t>0001327567-24-000040</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000035/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
         </is>
       </c>
     </row>
@@ -6773,7 +6801,7 @@
         </is>
       </c>
       <c r="C108" s="2" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
@@ -6781,16 +6809,16 @@
         </is>
       </c>
       <c r="E108" s="27" t="n">
-        <v>286500000</v>
+        <v>286000000</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>0001327567-24-000040</t>
+          <t>0001327567-25-000035</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000035/</t>
         </is>
       </c>
     </row>
@@ -6806,7 +6834,7 @@
         </is>
       </c>
       <c r="C109" s="2" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
@@ -6814,16 +6842,16 @@
         </is>
       </c>
       <c r="E109" s="27" t="n">
-        <v>2138800000</v>
+        <v>2139000000</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>0001327567-24-000040</t>
+          <t>0001327567-25-000035</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000035/</t>
         </is>
       </c>
     </row>
@@ -6839,7 +6867,7 @@
         </is>
       </c>
       <c r="C110" s="2" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
@@ -6847,16 +6875,16 @@
         </is>
       </c>
       <c r="E110" s="27" t="n">
-        <v>2139000000</v>
+        <v>2138800000</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>0001327567-25-000035</t>
+          <t>0001327567-24-000040</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000035/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
         </is>
       </c>
     </row>

</xml_diff>